<commit_message>
feat(combat): G07-P1-B5 execute action and break scheduling
</commit_message>
<xml_diff>
--- a/config/data/Operation.xlsx
+++ b/config/data/Operation.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1833,6 +1833,120 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="B38" t="n">
+        <v>24701</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>goal07.probe.operation.force-break</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>14001</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Fault</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EventSnapshot</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Rollback</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>{"type":"Break","element":"Fire"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="n">
+        <v>24702</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>goal07.probe.operation.delay-action</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>24051</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Fault</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Rollback</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>{"type":"DelayAction","amount_expression_id":24309}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="n">
+        <v>24703</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>goal07.probe.operation.grant-extra-turn</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>24051</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Fault</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Rollback</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>{"type":"GrantExtraTurn","actor_selector_id":24051}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>